<commit_message>
Jewelry lead run results
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011EVb4KaNaj6AQ86xbNTbBs
</commit_message>
<xml_diff>
--- a/leadrun_jewelry/jewelry_qualified.xlsx
+++ b/leadrun_jewelry/jewelry_qualified.xlsx
@@ -642,8 +642,16 @@
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Corey Friedman</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Featured On About Page</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>https://coreyfriedman.com</t>
@@ -2978,8 +2986,16 @@
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Bob Cohen</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Featured On About Page</t>
+        </is>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
           <t>https://cohensjewelers.com</t>
@@ -4830,8 +4846,16 @@
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Ricardo Basta</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Featured On About Page</t>
+        </is>
+      </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
           <t>https://ricardobasta.com</t>
@@ -4942,8 +4966,16 @@
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Phyllis Incidis</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
           <t>https://siorojewelry.com</t>
@@ -5146,8 +5178,16 @@
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
-      <c r="H44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Stephen Forward</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Featured On About Page</t>
+        </is>
+      </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
           <t>https://beverleyr.com</t>
@@ -5906,8 +5946,16 @@
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Stan Razny</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
           <t>https://www.razny.com</t>
@@ -6678,8 +6726,16 @@
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Lance Deutsch</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Featured On About Page</t>
+        </is>
+      </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
           <t>https://www.deutschhouston.com</t>
@@ -7338,8 +7394,16 @@
         </is>
       </c>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Matthew Cooper</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Featured On About Page</t>
+        </is>
+      </c>
       <c r="I64" s="2" t="inlineStr">
         <is>
           <t>https://www.kanonn.net</t>
@@ -11782,8 +11846,16 @@
         </is>
       </c>
       <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
-      <c r="H106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Andrea Hill</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
       <c r="I106" s="2" t="inlineStr">
         <is>
           <t>https://www.atlantajewelryshow.com</t>
@@ -12846,8 +12918,16 @@
         </is>
       </c>
       <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr"/>
-      <c r="H116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Ron DeSumma</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
           <t>https://desummaandwexler.com</t>
@@ -13170,8 +13250,16 @@
         </is>
       </c>
       <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
-      <c r="H119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Kenyatta Black</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
       <c r="I119" s="2" t="inlineStr">
         <is>
           <t>https://www.philadelphiadiamondco.com</t>
@@ -14562,8 +14650,16 @@
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
-      <c r="G132" t="inlineStr"/>
-      <c r="H132" t="inlineStr"/>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Lia Davis Lombara</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
       <c r="I132" s="2" t="inlineStr">
         <is>
           <t>https://colbydavisofboston.com</t>
@@ -15699,7 +15795,7 @@
         <v>20</v>
       </c>
       <c r="F2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -15726,7 +15822,7 @@
         <v>22</v>
       </c>
       <c r="F3" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -15753,7 +15849,7 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -15780,7 +15876,7 @@
         <v>20</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -15861,7 +15957,7 @@
         <v>11</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
@@ -15888,7 +15984,7 @@
         <v>7</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -15942,7 +16038,7 @@
         <v>9</v>
       </c>
       <c r="F11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -15969,7 +16065,7 @@
         <v>136</v>
       </c>
       <c r="F12" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
@@ -16113,7 +16209,7 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>2026-10-13T19:16:28+05:30</t>
+          <t>2026-10-13T21:22:07+05:30</t>
         </is>
       </c>
     </row>

</xml_diff>